<commit_message>
Atualiza relatorio e configuracoes do gitignore
</commit_message>
<xml_diff>
--- a/relatorio_estudantes.xlsx
+++ b/relatorio_estudantes.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Estudantes" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -540,6 +540,32 @@
       <c r="E5" t="inlineStr">
         <is>
           <t>Não</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HELEN KELLER
+</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>venezuela</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nao</t>
         </is>
       </c>
     </row>

</xml_diff>